<commit_message>
cleaning up the base server
</commit_message>
<xml_diff>
--- a/base-mcp/database.xlsx
+++ b/base-mcp/database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amdcloud-my.sharepoint.com/personal/amysuo12_amd_com/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{226E0D31-C854-41BF-88CF-AAD78557D3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{226E0D31-C854-41BF-88CF-AAD78557D3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{715FDA0D-4626-4BBC-9566-76271718775A}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="8170" xr2:uid="{411DEED7-4BA9-47AA-89A8-99ECA8351376}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{411DEED7-4BA9-47AA-89A8-99ECA8351376}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,22 +56,22 @@
     <t>dsadw</t>
   </si>
   <si>
-    <t>h</t>
-  </si>
-  <si>
     <t>jados</t>
   </si>
   <si>
-    <t>y</t>
-  </si>
-  <si>
     <t>asnds</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
     <t>asdaw</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>mary</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -479,10 +479,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
       </c>
       <c r="D3">
         <v>132030</v>
@@ -493,10 +493,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D4">
         <v>2130921</v>
@@ -507,10 +507,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5">
         <v>123531</v>

</xml_diff>